<commit_message>
docs(order-management): finalize 24.14 scope — 7/7 deliverable, Order.notes reserved, blank-at-checkout resolved
</commit_message>
<xml_diff>
--- a/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
+++ b/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>7 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 0 out of scope.</t>
+          <t>7 requirement(s) to implement here — all 7 confirmed Deliverable with the human on 2026-07-02 (per-item walkthrough; Confluence sync check passed). 0 covered elsewhere, 0 out of scope. Confirmed build scope: 24.14-a…g. Jira: SBE-1138 (In Progress, Prantik Saha).</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Story 24.14 asks for an admin-only "Notes" surface on the Order Details page where admins add/edit Internal Notes, a Payment Memo, Invoice Notes / PO Number, and Additional Terms &amp; Conditions on an order, with every note addition/modification captured in a permanent, non-editable, backend-enforced audit trail. Re-verification against admin-backend-api confirms every supporting primitive is built and the cited evidence is accurate: the Order model exists with a free-text `notes` column (schema.prisma:1570); the append-only AdminAuditLog model + AdminAuditService.record()/recordMany() pattern is fully implemented (monthly-partitioned, transaction-aware) and already writes order-scoped entries via the checkout flow (entity enum value `order` at schema:2193, used in checkout.service.ts); and the account-history-notes module is a working, identical template (transactional note-column update + audit write). Three of the four note fields (payment_memo, invoice_note/PO, additional_terms) are not yet columns on Order, but invoice_note and additional_terms already exist verbatim on Cart, and adding plain scalar columns plus the net-new admin endpoints is straightforward in the migration source-of-truth repo. Overall verdict: fully Deliverable now. The only correction to the prior analysis is endpoint pathing — the codebase uses bare resource-name controllers under a global `api/v1` prefix (no `/admin` segment).</t>
+          <t>Admin-only Notes surface on Order Details: Internal Notes, Payment Memo, Invoice Note/PO Number, Additional Terms, each change captured in the permanent append-only AdminAuditLog. All primitives verified on dev 2026-07-02. KEY CORRECTION: Order.notes cannot be reused — it is the exhibitor checkout idempotency-key store (cart.service.ts:1277/:1541, payments.service.ts:213/:465, 24h duplicate-charge protection) — so 24.14-a gets a net-new internal_notes column. One migration adds four nullable columns to orders: internal_notes Text, payment_memo Text, invoice_note VarChar(255) (copied from Cart), additional_terms Text (copied from Cart) — created blank at checkout (resolved 2026-07-02, no Cart seeding). API surface = single endpoint pair GET+PATCH /api/v1/orders/:id/notes on the shipped orders module (per-field audit via recordMany in one transaction; permissions orders.notes.read/update documented in Swagger). Fully Deliverable now, zero external dependencies, no open questions.</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope finalized with the human 2026-07-02 (all 7 Deliverable). SBE ticket: SBE-1138 (In Progress, Prantik Saha).</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-02)</t>
         </is>
       </c>
     </row>
@@ -816,18 +816,18 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The Order model already carries a free-text `notes` column (verified). No admin write-path/endpoint exists yet (no Order Management controller exists at all — net-new for the whole epic), so a net-new admin endpoint must be built on top of the existing Order model and admin guards. Building that endpoint on a built primitive is Deliverable.</t>
+          <t>Confirmed 2026-07-02 WITH DELIVERY CORRECTION: Order.notes must NOT be reused — it is the exhibitor checkout idempotency-key store (written as 'idempotency_key:&lt;key&gt;' at order creation, substring-matched for 24h replay/duplicate-charge protection in BOTH exhibitor checkout paths); admin overwrite would break duplicate-order protection and the tab would render machine tags. Delivery = net-new internal_notes String? @db.Text column + shared GET/PATCH /orders/:id/notes on the shipped orders module.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1570 (Order.notes String? @db.Text — confirmed); src/auth/guards/roles.guard.ts, src/auth/decorators/permissions.decorator.ts (admin enforcement, confirmed present)</t>
+          <t>exhibitor-backend-api/src/cart/services/cart.service.ts:1277 (notes write), :1541 (contains replay lookup); src/payments/services/payments.service.ts:213 (write), :465 (lookup); src/cart/helpers/cart.helpers.ts:11 (buildIdempotencyKey); admin schema.prisma:1570 (Order.notes — leave untouched); other 3 repos: zero Order.notes references</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>[C5 cross-reference] OWNER — build here (GET + PATCH /api/v1/orders/:id/notes — the single read/writ…); reused by other stories in this cluster.</t>
+          <t>[C5 cross-reference] OWNER — build here (GET + PATCH /api/v1/orders/:id/notes — the single read/write pair); reused by other stories in this cluster. CORRECTION 2026-07-02: net-new internal_notes column — Order.notes is reserved (exhibitor idempotency-key store).</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started — scope confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Confirmed no payment_memo column exists on Order and no payment-memo write-path exists anywhere in src/ (grep returned nothing). The story owns adding a plain scalar column to the existing Order model (admin-backend-api is the migration source of truth) plus the net-new endpoint. All supporting primitives (Order model, admin guards, audit service) are built, so this is Deliverable.</t>
+          <t>Confirmed 2026-07-02. No payment_memo column on Order, no write path in any of the 5 repos (grep clean). Decision: payment_memo String? @db.Text (Text over VarChar, per human) in this story's migration, exposed via the shared notes endpoints. Order-level — distinct from story 24.8's planned payment_transactions.payment_memo (installment-level). Resolved 2026-07-02: created blank at checkout (no Cart seeding).</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1540-1604 (Order model — verified no payment_memo field); grep 'payment_memo' across schema and src/ → no matches</t>
+          <t>admin-backend-api/prisma/schema.prisma:1540-1604 (Order model — no payment_memo); grep 'payment_memo' across all 5 repos → no matches</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -900,7 +900,7 @@
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started — scope confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -932,12 +932,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Order has no invoice_note / po_number column (verified), but the identical field already exists on the Cart model labelled 'Invoice Note / PO Number', proving the pattern and DTO/validation shape. Adding the column to Order plus the admin endpoint is net-new build on existing primitives.</t>
+          <t>Confirmed 2026-07-02. Decision: ONE combined column (not separate invoice_note + po_number), copying Cart.invoice_note verbatim — String? @db.VarChar(255), comment 'Invoice Note / PO Number' — one shape for the same field across the domain; DTO/validation proven by the existing Cart write path. Resolved 2026-07-02: created blank at checkout (no Cart seeding).</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2811 (Cart.invoice_note String? — comment 'Invoice Note / PO Number'); src/admin/cart/dto/update-cart.dto.ts:85 + cart.service.ts:359 (existing write-path on Cart); Order model 1540-1604 has no such column</t>
+          <t>admin-backend-api/prisma/schema.prisma:2853 (Cart.invoice_note template); src/admin/cart/dto/update-cart.dto.ts:85 + cart.service.ts:359 (existing Cart write-path); Order model 1540-1604 has no such column</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -958,7 +958,7 @@
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started — scope confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -990,12 +990,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Order has no additional_terms column (verified); the same field already exists on Cart (additional_terms Text) and is already consumed by agreement-document.service.ts, proving the field and its handling. Adding the column to Order plus the admin endpoint is net-new build on existing primitives.</t>
+          <t>Confirmed 2026-07-02. Copy Cart.additional_terms verbatim — String? @db.Text, comment 'Additional Terms &amp; Conditions'; semantics proven by the existing consumer (agreement-document generator). Resolved 2026-07-02: created blank at checkout (no Cart seeding).</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2812 (Cart.additional_terms String? @db.Text — comment 'Additional Terms &amp; Conditions'); src/admin/cart/services/agreement-document.service.ts:112 (existing consumer); Order model 1540-1604 lacks it</t>
+          <t>admin-backend-api/prisma/schema.prisma:2854 (Cart.additional_terms template); src/admin/cart/services/agreement-document.service.ts:112 (existing consumer); Order model 1540-1604 lacks it</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started — scope confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Verified: the append-only AdminAuditLog model + AdminAuditService.record()/recordMany() pattern is fully implemented, monthly-partitioned, transaction-aware, and already writes order-scoped entries. The enum AdminAuditEntityType includes `order` and it is used in the checkout flow today. No update/delete endpoints exist on audit logs (permanent + non-editable — the controller exposes only GET routes). New note endpoints just call audit.record() inside the same Prisma transaction, exactly like account-history-notes.service.ts.</t>
+          <t>Confirmed 2026-07-02. Append-only AdminAuditLog (monthly-partitioned) + tx-aware record()/recordMany() fully built; enum 'order' already used by admin checkout. Non-editable is structural (audit controller is GET-only). Delivery = one recordMany call inside the PATCH $transaction — one entry per changed field with previous/new snapshots, per the account-history-notes pattern. Display = existing GET /logs/admin-audit (zero new endpoints).</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2193 (enum value `order`), :2209-2226 (AdminAuditLog @@id([id,created_at]), append-only/partitioned); src/admin/common/audit/admin-audit.service.ts:30-48 (record, tx-aware); src/admin/cart/services/checkout.service.ts (AdminAuditEntityType.order audit write, verified ~line 329); src/admin/account-history-notes/account-history-notes.service.ts:32-49 (note-update + audit-in-transaction pattern)</t>
+          <t>admin schema.prisma:2193 (enum 'order'), :2209-2226 (AdminAuditLog append-only/partitioned); src/admin/common/audit/admin-audit.service.ts:30-48 (record, tx-aware) + recordMany; src/admin/account-history-notes/account-history-notes.service.ts:25-55 (template); src/admin/audit-log/admin-audit-log.controller.ts (GET-only)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started — scope confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>These endpoints live in admin-backend-api (admin-only surface) behind JWT + roles + permissions guards (all verified present). Enforcement is just guard/decorator application on the net-new controller, matching every existing admin controller (e.g. @Permissions on admin-audit-log.controller.ts:30). The companion exhibitor-facing Order History (Epic 13) simply must not select these columns — that is the other epic's concern, not a blocker here.</t>
+          <t>Confirmed 2026-07-02. Routes behind the global JWT + roles + @Permissions stack (app.module.ts:86-91). Delivery = orders.notes.read / orders.notes.update permission seeds + decorators; permission keys documented on the Swagger route docs (human addition 2026-07-02). Customer side structurally safe: exhibitor uses frozen SELECT constants and its schema.prisma won't carry the new columns.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/auth/guards/jwt-auth.guard.ts, roles.guard.ts (confirmed); src/auth/decorators/permissions.decorator.ts; src/admin/audit-log/admin-audit-log.controller.ts:30 (@Permissions('logs.admin-audit.list') guard pattern)</t>
+          <t>src/auth/guards/jwt-auth.guard.ts, roles.guard.ts; src/auth/decorators/permissions.decorator.ts; permission.seeder.ts ~:1203 ('orders' block precedent); role.seeder.ts:178 (grant precedent)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started — scope confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>All logic (note persistence + audit write) is implemented server-side in admin-backend-api services/controllers, mirroring the existing account-history-notes module which updates a note column and records an audit entry atomically in a Prisma $transaction. Verified end-to-end.</t>
+          <t>Confirmed 2026-07-02. AC umbrella over a–e mechanics: DTO validation + order-exists/soft-delete 404 in the service layer; note write + per-field audit entries in one Prisma $transaction (failed audit write rolls back the note change); audit permanence is DB/API-structural. No build beyond the agreed endpoints.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/account-history-notes/account-history-notes.service.ts:25-55 (backend note update + transactional audit, verified); src/admin/common/audit/admin-audit.service.ts:30-48</t>
+          <t>src/admin/account-history-notes/account-history-notes.service.ts:25-55 (transactional template); src/admin/common/audit/admin-audit.service.ts:30-48</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started — scope confirmed 2026-07-02</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Return the order's internal notes, payment memo, invoice/PO note, and additional terms for the admin Notes tab.</t>
+          <t>Return the order's notes bundle — internal_notes, payment_memo, invoice_note, additional_terms — for the admin Notes tab. Permission: orders.notes.read (documented in the route's Swagger docs).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Add/edit internal notes, payment memo, invoice/PO note, and additional terms in one transaction; AdminAuditLog per change.</t>
+          <t>Update any subset of the four fields in one $transaction (all DTO fields optional; omitted fields untouched); one AdminAuditLog entry per changed field via recordMany. Permission: orders.notes.update (documented in the route's Swagger docs).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>24.6 — Order Details notes/invoice-note/terms editing (24.6-c/e/f) reuses this canonical write path.</t>
+          <t>24.6 — Order Details notes/invoice-note/terms editing (24.6-c/e/f) reuses this canonical write path; 24.6-d flips Not Deliverable → Deliverable when payment_memo lands.</t>
         </is>
       </c>
     </row>
@@ -1372,22 +1372,24 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>At checkout the Cart already holds invoice_note and additional_terms (and the checkout flow creates the Order from a cart), but the new Order-level columns are net-new. The spec only describes admins entering these fresh on the order's Notes tab and says nothing about deriving them from the cart, so it is unsettled whether checkout.service should seed the new Order columns from the cart at order-creation time (like other billing snapshots) or leave them blank for the admin to fill in.</t>
+          <t>None — register empty. The single item (cart-seeding of the new Order columns) was resolved with the human on 2026-07-02; decision recorded in the 24.14-b/c/d Requirements rows per the doc-format rule.</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>OPEN — for team discussion</t>
+          <t>RESOLVED (2026-07-02)</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Current direction (2026-07-01): (pending). Leaning toward leaving the new Order columns blank at order-creation (admin fills them on the Notes tab); team to confirm whether checkout should snapshot the Cart values instead. No code until answered.</t>
+          <t>Leave the new Order columns blank at order creation — the spec frames these as admin-entered fields on the Notes tab; no checkout write-path changes in any repo.</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1476,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>— (not started). No SBE ticket / PR / Swagger tag yet.</t>
+          <t>— (not started). SBE ticket: SBE-1138 (In Progress, Prantik Saha). No PR / Swagger tag yet.</t>
         </is>
       </c>
     </row>
@@ -1486,7 +1488,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Not yet implemented — analysis/feasibility stage only. Every in-scope requirement is ◻ Not started.</t>
+          <t>Scope finalized with the human 2026-07-02 — all 7 requirements confirmed Deliverable (per-item walkthrough; Confluence sync check passed). Implementation not started; every requirement ◻ Not started.</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1500,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Internal Notes admin GET/PATCH over existing Order.notes column.</t>
+          <t>◻ Not started — Internal Notes GET/PATCH via NET-NEW internal_notes Text column (Order.notes reserved: exhibitor checkout idempotency-key store)</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1512,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Payment Memo; needs net-new payment_memo scalar column on Order + endpoint.</t>
+          <t>◻ Not started — Payment Memo; net-new payment_memo Text column on Order (distinct from 24.8's payment_transactions.payment_memo)</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1524,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Invoice Notes / PO Number; needs net-new column on Order (pattern exists on Cart).</t>
+          <t>◻ Not started — Invoice Notes / PO Number; net-new invoice_note VarChar(255), one combined column copied from Cart.invoice_note</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1536,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Additional Terms &amp; Conditions; needs net-new column on Order (pattern exists on Cart).</t>
+          <t>◻ Not started — Additional Terms; net-new additional_terms Text copied from Cart.additional_terms</t>
         </is>
       </c>
     </row>
@@ -1577,12 +1579,12 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Open decision — Cart-seeding</t>
+          <t>Resolved decision — Cart-seeding</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Whether checkout.service seeds the net-new Order invoice_note/additional_terms/payment_memo columns from the Cart at order-creation, or leaves them blank for the admin. No code until answered.</t>
+          <t>RESOLVED 2026-07-02: new Order note columns are created blank at checkout (no seeding from Cart); admin fills them on the Notes tab. No checkout write-path changes in any repo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): record 24.14 implementation status — built on feature/SBE-1125, merge deferred
</commit_message>
<xml_diff>
--- a/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
+++ b/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>7 requirement(s) to implement here — all 7 confirmed Deliverable with the human on 2026-07-02 (per-item walkthrough; Confluence sync check passed). 0 covered elsewhere, 0 out of scope. Confirmed build scope: 24.14-a…g. Jira: SBE-1138 (In Progress, Prantik Saha).</t>
+          <t>All 7 requirements confirmed Deliverable AND implemented 2026-07-02 on feature/SBE-1125 (admin 8dbc089, pushed). PR/pipeline/merge deferred — team not merging to dev right now. Jira: SBE-1138 (In Progress, Prantik Saha).</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Not started — scope finalized with the human 2026-07-02 (all 7 Deliverable). SBE ticket: SBE-1138 (In Progress, Prantik Saha).</t>
+          <t>Implemented 2026-07-02 — pre-push gate 8/8, 2736 tests green, live smoke 15/15, Swagger proven. PR not raised (merge deferred).</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>feature/SBE-1125 (admin-backend-api; + same-named schema-sync branches in the 4 sibling repos)</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>admin 8dbc089 feat(SBE-1138); siblings 3d5fc2f / 7a2b359 / 9166612 / 1018402 chore(SBE-1138)</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>— not raised (merge to dev deferred by team, 2026-07-02); pipelines are PR-triggered so none run yet</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — scope confirmed 2026-07-02</t>
+          <t>✅ Implemented 2026-07-02 (feature/SBE-1125, 8dbc089; PR pending)</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="L3" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — scope confirmed 2026-07-02</t>
+          <t>✅ Implemented 2026-07-02 (feature/SBE-1125, 8dbc089; PR pending)</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — scope confirmed 2026-07-02</t>
+          <t>✅ Implemented 2026-07-02 (feature/SBE-1125, 8dbc089; PR pending)</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="L5" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — scope confirmed 2026-07-02</t>
+          <t>✅ Implemented 2026-07-02 (feature/SBE-1125, 8dbc089; PR pending)</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — scope confirmed 2026-07-02</t>
+          <t>✅ Implemented 2026-07-02 (feature/SBE-1125, 8dbc089; PR pending)</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — scope confirmed 2026-07-02</t>
+          <t>✅ Implemented 2026-07-02 (feature/SBE-1125, 8dbc089; PR pending)</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — scope confirmed 2026-07-02</t>
+          <t>✅ Implemented 2026-07-02 (feature/SBE-1125, 8dbc089; PR pending)</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>— (not started). SBE ticket: SBE-1138 (In Progress, Prantik Saha). No PR / Swagger tag yet.</t>
+          <t>feature/SBE-1125 (admin; renamed from bare SBE-1125, rebased onto dev f1a9c67). Commits: admin 8dbc089 (+716, 11 files); sibling schema syncs 3d5fc2f/7a2b359/9166612/1018402 on same-named branches. PR: not raised — merge deferred; no pipeline run yet.</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>Scope finalized with the human 2026-07-02 — all 7 requirements confirmed Deliverable (per-item walkthrough; Confluence sync check passed). Implementation not started; every requirement ◻ Not started.</t>
+          <t>IMPLEMENTED 2026-07-02, all 7 reqs. Gates: pre-push 8/8, scoped tests 69, full suite 2736, coverage 94.67%/95.58%; live smoke 15/15 (idempotency tag intact, audit rows exact, negatives, teardown); Swagger routes + permission keys proven in OpenAPI JSON. Lifecycle remaining: 5 PRs vs dev, pipeline/Sonar to green, merge. Pre-existing gap flagged: no role has logs.admin-audit.list → audit UI 403.</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Internal Notes GET/PATCH via NET-NEW internal_notes Text column (Order.notes reserved: exhibitor checkout idempotency-key store)</t>
+          <t>✅ Implemented — internal_notes Text; Order.notes untouched (smoke-proven)</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Payment Memo; net-new payment_memo Text column on Order (distinct from 24.8's payment_transactions.payment_memo)</t>
+          <t>✅ Implemented — payment_memo Text on Order</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Invoice Notes / PO Number; net-new invoice_note VarChar(255), one combined column copied from Cart.invoice_note</t>
+          <t>✅ Implemented — invoice_note VarChar(255), one combined column</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Additional Terms; net-new additional_terms Text copied from Cart.additional_terms</t>
+          <t>✅ Implemented — additional_terms Text</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Permanent non-editable audit trail via AdminAuditService.record() in the same Prisma transaction.</t>
+          <t>✅ Implemented — per-changed-field recordMany in the PATCH transaction (psql-verified)</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Admin-only visibility via JWT + roles + @Permissions guards on the net-new controller.</t>
+          <t>✅ Implemented — perms seeded/granted + documented in Swagger; siblings carry columns schema-only</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>◻ Not started — Backend-enforced transactional note update + audit, per account-history-notes pattern.</t>
+          <t>✅ Implemented — transactional write + audit, rollback unit-tested</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.14 PRs raised — pipelines + Sonar green x5, merge pending
</commit_message>
<xml_diff>
--- a/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
+++ b/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>All 7 requirements confirmed Deliverable AND implemented 2026-07-02 on feature/SBE-1125 (admin 8dbc089, pushed). PR/pipeline/merge deferred — team not merging to dev right now. Jira: SBE-1138 (In Progress, Prantik Saha).</t>
+          <t>All 7 requirements confirmed Deliverable AND implemented 2026-07-02 on feature/SBE-1125 (admin 8dbc089, pushed). All 5 PRs raised 2026-07-02 — pipelines + SonarQube green; merge to dev pending team. Jira: SBE-1138 (In Progress, Prantik Saha).</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Implemented 2026-07-02 — pre-push gate 8/8, 2736 tests green, live smoke 15/15, Swagger proven. PR not raised (merge deferred).</t>
+          <t>Implemented 2026-07-02 — pre-push gate 8/8, 2736 tests green, live smoke 15/15, Swagger proven. PRs raised 2026-07-02, pipelines + Sonar green (merge pending).</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>— not raised (merge to dev deferred by team, 2026-07-02); pipelines are PR-triggered so none run yet</t>
+          <t>Raised 2026-07-02, all pipelines SUCCESSFUL + Sonar gate OK: admin PR#516 (#841) / exhibitor PR#284 (#410) / background-worker PR#25 (#35) / external-api PR#88 (#121) / pulse-broker PR#14 (#17). Merge pending team.</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>feature/SBE-1125 (admin; renamed from bare SBE-1125, rebased onto dev f1a9c67). Commits: admin 8dbc089 (+716, 11 files); sibling schema syncs 3d5fc2f/7a2b359/9166612/1018402 on same-named branches. PR: not raised — merge deferred; no pipeline run yet.</t>
+          <t>feature/SBE-1125 (admin; renamed from bare SBE-1125, rebased onto dev f1a9c67). Commits: admin 8dbc089 (+716, 11 files); sibling schema syncs 3d5fc2f/7a2b359/9166612/1018402 on same-named branches. PRs raised 2026-07-02: admin #516, exhibitor #284, bg-worker #25, external #88, pulse #14 — all pipelines SUCCESSFUL, Sonar gates OK; merge to dev pending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.14 merged to dev — story complete; flip 24.6-c/d/e/f to Deliverable, resolve payment-memo + notes-sourcing questions
</commit_message>
<xml_diff>
--- a/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
+++ b/order_management/24.14-internal-notes-and-administrative-information/24.14 - Internal Notes & Administrative Information.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>All 7 requirements confirmed Deliverable AND implemented 2026-07-02 on feature/SBE-1125 (admin 8dbc089, pushed). All 5 PRs raised 2026-07-02 — pipelines + SonarQube green; merge to dev pending team. Jira: SBE-1138 (In Progress, Prantik Saha).</t>
+          <t>All 7 requirements confirmed Deliverable AND implemented 2026-07-02 on feature/SBE-1125 (admin 8dbc089). All 5 PRs raised 2026-07-02, pipelines + SonarQube green, MERGED to dev 2026-07-03. STORY COMPLETE. Jira: SBE-1138.</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Implemented 2026-07-02 — pre-push gate 8/8, 2736 tests green, live smoke 15/15, Swagger proven. PRs raised 2026-07-02, pipelines + Sonar green (merge pending).</t>
+          <t>Implemented 2026-07-02 — pre-push gate 8/8, 2736 tests green, live smoke 15/15, Swagger proven. PRs raised 2026-07-02, pipelines + Sonar green; MERGED to dev 2026-07-03.</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Raised 2026-07-02, all pipelines SUCCESSFUL + Sonar gate OK: admin PR#516 (#841) / exhibitor PR#284 (#410) / background-worker PR#25 (#35) / external-api PR#88 (#121) / pulse-broker PR#14 (#17). Merge pending team.</t>
+          <t>MERGED to dev 2026-07-03 (all pipelines SUCCESSFUL + Sonar OK): admin PR#516 (merge 09a652d) / exhibitor PR#284 (8c70e36) / background-worker PR#25 (fbfcd8c) / external-api PR#88 (e585659) / pulse-broker PR#14 (ffd3e5a).</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>feature/SBE-1125 (admin; renamed from bare SBE-1125, rebased onto dev f1a9c67). Commits: admin 8dbc089 (+716, 11 files); sibling schema syncs 3d5fc2f/7a2b359/9166612/1018402 on same-named branches. PRs raised 2026-07-02: admin #516, exhibitor #284, bg-worker #25, external #88, pulse #14 — all pipelines SUCCESSFUL, Sonar gates OK; merge to dev pending.</t>
+          <t>feature/SBE-1125 (admin; rebased onto dev f1a9c67). Commits: admin 8dbc089 (+716, 11 files); sibling schema syncs 3d5fc2f/7a2b359/9166612/1018402. PRs raised 2026-07-02 (admin #516, exhibitor #284, bg-worker #25, external #88, pulse #14), all pipelines + Sonar green; MERGED to dev 2026-07-03. Story complete; 24.6-c/d/e/f verdicts flipped same day.</t>
         </is>
       </c>
     </row>

</xml_diff>